<commit_message>
fix: Expanded Relevo/Cambio de guardia window to 18:00 PM to correctly recognize tardanza in relevo block without false excess shift
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-22.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-22.xlsx
@@ -2144,117 +2144,121 @@
       <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>03208053</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>MORETO BERMEO</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>FRANCO</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>06:32</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="L18" s="10" t="inlineStr">
         <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q18" s="7" t="inlineStr">
+      <c r="M18" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" s="10" t="inlineStr">
         <is>
           <t>10:23</t>
         </is>
       </c>
-      <c r="R18" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S18" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T18" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="V18" s="7" t="inlineStr">
-        <is>
-          <t>Cambio de guardia</t>
-        </is>
-      </c>
-      <c r="W18" s="6" t="inlineStr"/>
+      <c r="R18" s="10" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S18" s="10" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T18" s="10" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U18" s="10" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V18" s="10" t="inlineStr">
+        <is>
+          <t>Salida anticipada</t>
+        </is>
+      </c>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>Salida anticipada (01:26)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -17840,7 +17844,7 @@
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S155" s="7" t="inlineStr">
@@ -17850,7 +17854,7 @@
       </c>
       <c r="T155" s="7" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U155" s="7" t="inlineStr">
@@ -17860,12 +17864,12 @@
       </c>
       <c r="V155" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada/Tardanza</t>
+          <t>Cambio de guardia/Tardanza</t>
         </is>
       </c>
       <c r="W155" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:13), Tardanza (00:33)</t>
+          <t>Tardanza (00:33)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Moved Tardanza column to Column R (right after Horas de Turno) and updated Excel layout
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-22.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-22.xlsx
@@ -641,22 +641,22 @@
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
+          <t>Tardanza</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
           <t>Exceso de Turno</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>Horas Extras</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>Total de Horas Adicionales</t>
-        </is>
-      </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>Tardanza</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
@@ -2348,22 +2348,22 @@
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S19" s="7" t="inlineStr">
+        <is>
           <t>01:56</t>
         </is>
       </c>
-      <c r="S19" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U19" s="7" t="inlineStr">
+        <is>
           <t>01:56</t>
-        </is>
-      </c>
-      <c r="U19" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:57</t>
         </is>
       </c>
       <c r="S31" s="7" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>00:57</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V31" s="7" t="inlineStr">
@@ -5654,17 +5654,17 @@
       </c>
       <c r="S48" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T48" s="7" t="inlineStr">
+        <is>
           <t>04:00</t>
         </is>
       </c>
-      <c r="T48" s="7" t="inlineStr">
+      <c r="U48" s="7" t="inlineStr">
         <is>
           <t>04:00</t>
-        </is>
-      </c>
-      <c r="U48" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V48" s="7" t="inlineStr">
@@ -5771,17 +5771,17 @@
       </c>
       <c r="S49" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T49" s="7" t="inlineStr">
+        <is>
           <t>03:53</t>
         </is>
       </c>
-      <c r="T49" s="7" t="inlineStr">
+      <c r="U49" s="7" t="inlineStr">
         <is>
           <t>03:53</t>
-        </is>
-      </c>
-      <c r="U49" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V49" s="7" t="inlineStr">
@@ -5888,17 +5888,17 @@
       </c>
       <c r="S50" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T50" s="7" t="inlineStr">
+        <is>
           <t>03:20</t>
         </is>
       </c>
-      <c r="T50" s="7" t="inlineStr">
+      <c r="U50" s="7" t="inlineStr">
         <is>
           <t>03:20</t>
-        </is>
-      </c>
-      <c r="U50" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V50" s="7" t="inlineStr">
@@ -6005,17 +6005,17 @@
       </c>
       <c r="S51" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T51" s="7" t="inlineStr">
+        <is>
           <t>04:50</t>
         </is>
       </c>
-      <c r="T51" s="7" t="inlineStr">
+      <c r="U51" s="7" t="inlineStr">
         <is>
           <t>04:50</t>
-        </is>
-      </c>
-      <c r="U51" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V51" s="7" t="inlineStr">
@@ -6908,22 +6908,22 @@
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S59" s="7" t="inlineStr">
+        <is>
           <t>00:56</t>
         </is>
       </c>
-      <c r="S59" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T59" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U59" s="7" t="inlineStr">
+        <is>
           <t>00:56</t>
-        </is>
-      </c>
-      <c r="U59" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V59" s="7" t="inlineStr">
@@ -7025,22 +7025,22 @@
       </c>
       <c r="R60" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S60" s="7" t="inlineStr">
+        <is>
           <t>01:14</t>
         </is>
       </c>
-      <c r="S60" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T60" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U60" s="7" t="inlineStr">
+        <is>
           <t>01:14</t>
-        </is>
-      </c>
-      <c r="U60" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V60" s="7" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="R61" s="10" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:03</t>
         </is>
       </c>
       <c r="S61" s="10" t="inlineStr">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="U61" s="10" t="inlineStr">
         <is>
-          <t>00:03</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V61" s="10" t="inlineStr">
@@ -7368,22 +7368,22 @@
       </c>
       <c r="R63" s="7" t="inlineStr">
         <is>
+          <t>00:02</t>
+        </is>
+      </c>
+      <c r="S63" s="7" t="inlineStr">
+        <is>
           <t>01:10</t>
         </is>
       </c>
-      <c r="S63" s="7" t="inlineStr">
+      <c r="T63" s="7" t="inlineStr">
         <is>
           <t>01:40</t>
         </is>
       </c>
-      <c r="T63" s="7" t="inlineStr">
+      <c r="U63" s="7" t="inlineStr">
         <is>
           <t>02:50</t>
-        </is>
-      </c>
-      <c r="U63" s="7" t="inlineStr">
-        <is>
-          <t>00:02</t>
         </is>
       </c>
       <c r="V63" s="7" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="R67" s="10" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:03</t>
         </is>
       </c>
       <c r="S67" s="10" t="inlineStr">
@@ -7835,7 +7835,7 @@
       </c>
       <c r="U67" s="10" t="inlineStr">
         <is>
-          <t>00:03</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V67" s="10" t="inlineStr">
@@ -8389,22 +8389,22 @@
       </c>
       <c r="R72" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S72" s="7" t="inlineStr">
+        <is>
           <t>02:42</t>
         </is>
       </c>
-      <c r="S72" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T72" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U72" s="7" t="inlineStr">
+        <is>
           <t>02:42</t>
-        </is>
-      </c>
-      <c r="U72" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V72" s="7" t="inlineStr">
@@ -8511,17 +8511,17 @@
       </c>
       <c r="S73" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T73" s="7" t="inlineStr">
+        <is>
           <t>02:32</t>
         </is>
       </c>
-      <c r="T73" s="7" t="inlineStr">
+      <c r="U73" s="7" t="inlineStr">
         <is>
           <t>02:32</t>
-        </is>
-      </c>
-      <c r="U73" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V73" s="7" t="inlineStr">
@@ -8623,22 +8623,22 @@
       </c>
       <c r="R74" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S74" s="7" t="inlineStr">
+        <is>
           <t>00:30</t>
         </is>
       </c>
-      <c r="S74" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T74" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U74" s="7" t="inlineStr">
+        <is>
           <t>00:30</t>
-        </is>
-      </c>
-      <c r="U74" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V74" s="7" t="inlineStr">
@@ -8966,22 +8966,22 @@
       </c>
       <c r="R77" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S77" s="7" t="inlineStr">
+        <is>
           <t>01:11</t>
         </is>
       </c>
-      <c r="S77" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T77" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U77" s="7" t="inlineStr">
+        <is>
           <t>01:11</t>
-        </is>
-      </c>
-      <c r="U77" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V77" s="7" t="inlineStr">
@@ -9083,22 +9083,22 @@
       </c>
       <c r="R78" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S78" s="7" t="inlineStr">
+        <is>
           <t>01:11</t>
         </is>
       </c>
-      <c r="S78" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T78" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U78" s="7" t="inlineStr">
+        <is>
           <t>01:11</t>
-        </is>
-      </c>
-      <c r="U78" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V78" s="7" t="inlineStr">
@@ -9200,22 +9200,22 @@
       </c>
       <c r="R79" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S79" s="7" t="inlineStr">
+        <is>
           <t>03:26</t>
         </is>
       </c>
-      <c r="S79" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T79" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U79" s="7" t="inlineStr">
+        <is>
           <t>03:26</t>
-        </is>
-      </c>
-      <c r="U79" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V79" s="7" t="inlineStr">
@@ -9317,22 +9317,22 @@
       </c>
       <c r="R80" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S80" s="7" t="inlineStr">
+        <is>
           <t>00:47</t>
         </is>
       </c>
-      <c r="S80" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T80" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U80" s="7" t="inlineStr">
+        <is>
           <t>00:47</t>
-        </is>
-      </c>
-      <c r="U80" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V80" s="7" t="inlineStr">
@@ -9656,7 +9656,7 @@
       </c>
       <c r="R83" s="10" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="S83" s="10" t="inlineStr">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="U83" s="10" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V83" s="10" t="inlineStr">
@@ -10112,22 +10112,22 @@
       </c>
       <c r="R87" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S87" s="7" t="inlineStr">
+        <is>
           <t>00:35</t>
         </is>
       </c>
-      <c r="S87" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T87" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U87" s="7" t="inlineStr">
+        <is>
           <t>00:35</t>
-        </is>
-      </c>
-      <c r="U87" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V87" s="7" t="inlineStr">
@@ -11020,22 +11020,22 @@
       </c>
       <c r="R95" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S95" s="7" t="inlineStr">
+        <is>
           <t>01:18</t>
         </is>
       </c>
-      <c r="S95" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T95" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U95" s="7" t="inlineStr">
+        <is>
           <t>01:18</t>
-        </is>
-      </c>
-      <c r="U95" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V95" s="7" t="inlineStr">
@@ -11137,22 +11137,22 @@
       </c>
       <c r="R96" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S96" s="7" t="inlineStr">
+        <is>
           <t>02:38</t>
         </is>
       </c>
-      <c r="S96" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T96" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U96" s="7" t="inlineStr">
+        <is>
           <t>02:38</t>
-        </is>
-      </c>
-      <c r="U96" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V96" s="7" t="inlineStr">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="R106" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:02</t>
         </is>
       </c>
       <c r="S106" s="7" t="inlineStr">
@@ -12286,7 +12286,7 @@
       </c>
       <c r="U106" s="7" t="inlineStr">
         <is>
-          <t>00:02</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V106" s="7" t="inlineStr">
@@ -12727,22 +12727,22 @@
       </c>
       <c r="R110" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S110" s="7" t="inlineStr">
+        <is>
           <t>01:17</t>
         </is>
       </c>
-      <c r="S110" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T110" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U110" s="7" t="inlineStr">
+        <is>
           <t>01:17</t>
-        </is>
-      </c>
-      <c r="U110" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V110" s="7" t="inlineStr">
@@ -12844,22 +12844,22 @@
       </c>
       <c r="R111" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S111" s="7" t="inlineStr">
+        <is>
           <t>02:38</t>
         </is>
       </c>
-      <c r="S111" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T111" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U111" s="7" t="inlineStr">
+        <is>
           <t>02:38</t>
-        </is>
-      </c>
-      <c r="U111" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V111" s="7" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
       <c r="R116" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:41</t>
         </is>
       </c>
       <c r="S116" s="7" t="inlineStr">
@@ -13428,7 +13428,7 @@
       </c>
       <c r="U116" s="7" t="inlineStr">
         <is>
-          <t>00:41</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V116" s="7" t="inlineStr">
@@ -14099,7 +14099,7 @@
       </c>
       <c r="R122" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>03:32</t>
         </is>
       </c>
       <c r="S122" s="7" t="inlineStr">
@@ -14114,7 +14114,7 @@
       </c>
       <c r="U122" s="7" t="inlineStr">
         <is>
-          <t>03:32</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V122" s="7" t="inlineStr">
@@ -17844,7 +17844,7 @@
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:33</t>
         </is>
       </c>
       <c r="S155" s="7" t="inlineStr">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="U155" s="7" t="inlineStr">
         <is>
-          <t>00:33</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V155" s="7" t="inlineStr">
@@ -20003,7 +20003,7 @@
       </c>
       <c r="R174" s="10" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:29</t>
         </is>
       </c>
       <c r="S174" s="10" t="inlineStr">
@@ -20018,7 +20018,7 @@
       </c>
       <c r="U174" s="10" t="inlineStr">
         <is>
-          <t>00:29</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V174" s="10" t="inlineStr">
@@ -20237,22 +20237,22 @@
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S176" s="7" t="inlineStr">
+        <is>
           <t>01:23</t>
         </is>
       </c>
-      <c r="S176" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T176" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U176" s="7" t="inlineStr">
+        <is>
           <t>01:23</t>
-        </is>
-      </c>
-      <c r="U176" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V176" s="7" t="inlineStr">
@@ -20806,7 +20806,7 @@
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:39</t>
         </is>
       </c>
       <c r="S181" s="7" t="inlineStr">
@@ -20821,7 +20821,7 @@
       </c>
       <c r="U181" s="7" t="inlineStr">
         <is>
-          <t>00:39</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V181" s="7" t="inlineStr">
@@ -21262,22 +21262,22 @@
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S185" s="7" t="inlineStr">
+        <is>
           <t>02:43</t>
         </is>
       </c>
-      <c r="S185" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T185" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U185" s="7" t="inlineStr">
+        <is>
           <t>02:43</t>
-        </is>
-      </c>
-      <c r="U185" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V185" s="7" t="inlineStr">
@@ -21375,7 +21375,7 @@
       </c>
       <c r="R186" s="10" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="S186" s="10" t="inlineStr">
@@ -21390,7 +21390,7 @@
       </c>
       <c r="U186" s="10" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V186" s="10" t="inlineStr">
@@ -21492,7 +21492,7 @@
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:32</t>
         </is>
       </c>
       <c r="S187" s="7" t="inlineStr">
@@ -21507,7 +21507,7 @@
       </c>
       <c r="U187" s="7" t="inlineStr">
         <is>
-          <t>00:32</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="V187" s="7" t="inlineStr">
@@ -23313,17 +23313,17 @@
       </c>
       <c r="S203" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T203" s="7" t="inlineStr">
+        <is>
           <t>02:43</t>
         </is>
       </c>
-      <c r="T203" s="7" t="inlineStr">
+      <c r="U203" s="7" t="inlineStr">
         <is>
           <t>02:43</t>
-        </is>
-      </c>
-      <c r="U203" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V203" s="7" t="inlineStr">
@@ -23430,17 +23430,17 @@
       </c>
       <c r="S204" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T204" s="7" t="inlineStr">
+        <is>
           <t>02:00</t>
         </is>
       </c>
-      <c r="T204" s="7" t="inlineStr">
+      <c r="U204" s="7" t="inlineStr">
         <is>
           <t>02:00</t>
-        </is>
-      </c>
-      <c r="U204" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V204" s="7" t="inlineStr">
@@ -24220,22 +24220,22 @@
       </c>
       <c r="R211" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S211" s="7" t="inlineStr">
+        <is>
           <t>00:35</t>
         </is>
       </c>
-      <c r="S211" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="T211" s="7" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U211" s="7" t="inlineStr">
+        <is>
           <t>00:35</t>
-        </is>
-      </c>
-      <c r="U211" s="7" t="inlineStr">
-        <is>
-          <t>00:00</t>
         </is>
       </c>
       <c r="V211" s="7" t="inlineStr">

</xml_diff>